<commit_message>
Update 	new file:   "HM_CHA06/Bai 10 X\303\242y d\341\273\261ng \341\273\251ng d\341\273\245ng h\341\273\215c m\303\241y an to\303\240n.pdf" 	new file:   HM_CHA06/Bai 7 Phan tich mang.pdf 	new file:   "HM_CHA06/Bai 8 H\341\273\215c m\303\241y v\303\240 an to\303\240n \341\273\251ng d\341\273\245ng web.pdf" 	new file:   "HM_CHA06/Bai 9 Mat ma v\303\240 privacy preserving ML.pdf" 	new file:   HM_CHA06/Emmanuel Tsukerman - Machine Learning for Cybersecurity Cookbook_ Over 80 recipes on how to implement machine learning algorithms for building security systems using Python-Packt Publishing (2019).pdf 	new file:   HM_CHA06/Machine-Learning-for-Cybersecurity-Cookbook 	new file:   HM_CHA06/baitaplon.py 	modified:   HM_CHA06/ds BTL3.2024-HV.xlsx
</commit_message>
<xml_diff>
--- a/HM_CHA06/ds BTL3.2024-HV.xlsx
+++ b/HM_CHA06/ds BTL3.2024-HV.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vitho\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Work\Github\KMA_CHAT10\HM_CHA06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE66B0A3-C117-4ADF-9501-37904BE3CFA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{212A7059-611E-4957-AA65-F93456F40117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DS" sheetId="2" r:id="rId1"/>
@@ -645,15 +645,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C28"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.21875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="63.88671875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="63.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="32" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="1"/>
+    <col min="4" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="37.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>1</v>
       </c>
@@ -664,7 +664,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="27.6" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -675,7 +675,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -686,7 +686,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -697,7 +697,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="34.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -708,7 +708,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -719,7 +719,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="37.200000000000003" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="37.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -730,7 +730,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="35.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="35.450000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -741,7 +741,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -752,7 +752,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -763,7 +763,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -774,7 +774,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -785,7 +785,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="44.4" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="44.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -796,7 +796,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -807,7 +807,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="43.2" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="43.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -818,7 +818,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -829,7 +829,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -840,7 +840,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="46.8" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" ht="46.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -851,7 +851,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -862,7 +862,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="58.8" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" ht="58.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -873,7 +873,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="58.8" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" ht="58.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -884,7 +884,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -895,7 +895,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -906,7 +906,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -917,7 +917,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -928,7 +928,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -939,7 +939,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="36" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -950,7 +950,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>

</xml_diff>